<commit_message>
fix: use limit orders on Day1 and Day2
</commit_message>
<xml_diff>
--- a/docs/google_sheet_pipeline_template.xlsx
+++ b/docs/google_sheet_pipeline_template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="Rea063df3d77f4e6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="2" r:id="Rf661295372214d99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="程式輸入" sheetId="3" r:id="Rb74cb38c900b4410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每週計畫" sheetId="4" r:id="Rb19f24f2387f438d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="執行紀錄" sheetId="5" r:id="R74b9839ea2a7447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日確認" sheetId="6" r:id="R2a1d1869ccd44fef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="檢查" sheetId="7" r:id="R2912ea59d97445b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="R733fff61dfe849c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="2" r:id="Rece67f5d34b0492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="程式輸入" sheetId="3" r:id="R50cd6c41d9cb4bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每週計畫" sheetId="4" r:id="R7f51175e53584308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="執行紀錄" sheetId="5" r:id="R158d0b184ced45d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日確認" sheetId="6" r:id="R7d635e10d38a4319"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="檢查" sheetId="7" r:id="Red53573f76d942ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -507,7 +507,7 @@
         <x:v>Day1</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>Generate orders; enter actual fills in filled_price on the execution log.</x:v>
+        <x:v>Generate LIMIT orders; enter actual fills in filled_price on the execution log.</x:v>
       </x:c>
       <x:c r="C5" s="12"/>
       <x:c r="D5" s="12"/>
@@ -644,13 +644,13 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>market_immediate_rule</x:v>
+        <x:v>day1_day2_order_type</x:v>
       </x:c>
       <x:c r="B5" s="19" t="str">
-        <x:v>calculated_limit &gt;= current_price</x:v>
+        <x:v>LIMIT</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Switch to MARKET when true</x:v>
+        <x:v>Always preserve the maximum buy-price cap</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>